<commit_message>
Fixed errors in the data
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/app_detail.xlsx
+++ b/mosip_master/xlsx/app_detail.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\Sao-Tome-mosip-master\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\eclipse-workspace\mosip-data\mosip_master\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83BA3C41-28FD-49EA-B976-C1ACE5F4E6B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547FA29B-669C-4911-85C4-E9B99CE68DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="38">
   <si>
     <t>lang_code</t>
   </si>
@@ -136,6 +136,9 @@
   </si>
   <si>
     <t>Web portal for Post ID generation services</t>
+  </si>
+  <si>
+    <t>Portal Residente</t>
   </si>
 </sst>
 </file>
@@ -601,7 +604,7 @@
         <v>10011</v>
       </c>
       <c r="C7" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>

</xml_diff>